<commit_message>
Stage 8 review fixes: B-028
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2026/BW26_0401/Run_sheets/BW26_0401_RUN04.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2026/BW26_0401/Run_sheets/BW26_0401_RUN04.xlsx
@@ -184,7 +184,7 @@
   <commentList>
     <comment ref="E6" authorId="0" shapeId="0">
       <text>
-        <t>Quinidine control drifted at the start of the second plate set. In range, but I want the historical check repeated before the report.</t>
+        <t>Complete the control-acceptance review from the original run sheets before the signed report is released.</t>
       </text>
     </comment>
   </commentList>
@@ -491,7 +491,8 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BW26_0401 run sheet 04: 5-isoform CYP inhibition (INTERIM)</t>
+          <t>Brindlewythe Biosciences Ltd, a Tarnovell company
+BW26_0401 run sheet 04: 5-isoform CYP inhibition (INTERIM)</t>
         </is>
       </c>
     </row>
@@ -558,7 +559,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Compounds on run</t>
+          <t>Compounds on project</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -580,12 +581,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Runs</t>
+          <t>Study start / interim</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 to 24/09/2026</t>
+          <t>14/09/2026 / 24/09/2026</t>
         </is>
       </c>
     </row>
@@ -622,7 +623,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Recovery checked per sample card. Blank rows below are for the repeat.</t>
+          <t>Poorly recovered sample repeat open. Original sample cards identify the sample; blank rows below await reconciliation.</t>
         </is>
       </c>
     </row>
@@ -684,7 +685,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plate acceptance</t>
+          <t>Plate acceptance (INTERIM)</t>
         </is>
       </c>
     </row>
@@ -711,7 +712,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Review record</t>
         </is>
       </c>
     </row>
@@ -734,7 +735,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Original run sheets</t>
         </is>
       </c>
     </row>
@@ -757,7 +758,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Original run sheets</t>
         </is>
       </c>
     </row>
@@ -780,7 +781,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Original run sheets</t>
         </is>
       </c>
     </row>
@@ -803,7 +804,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Original run sheets</t>
         </is>
       </c>
     </row>
@@ -826,7 +827,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Original run sheets</t>
         </is>
       </c>
     </row>
@@ -834,7 +835,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Acceptance: control IC50 within the historical range for each isoform on every plate.</t>
+          <t>Control IC50s and historical reference values are shown for review. Consult original run sheets for acceptance limits and plate-level decisions; closeness to a reference value alone does not establish acceptance.</t>
         </is>
       </c>
     </row>
@@ -865,14 +866,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CYP inhibition, % at 10 µM, 40 compounds (interim)</t>
+          <t>CYP inhibition, % at 10 µM: partial interim table</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Negative values are within assay noise. Partial recovery samples are marked in the sample recovery tracker on the run sheet.</t>
+          <t>Duplicate incubations; mean reported. Negative values indicate no inhibition. Only the reported compound rows are shown; the sample recovery tracker awaits reconciliation.</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1349,7 +1350,8 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Interim summary</t>
+          <t>Brindlewythe Biosciences Ltd, a Tarnovell company
+Interim summary</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1380,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Compounds &gt;50% inhibition on at least one isoform</t>
+          <t>Project benchmark: compounds &gt;50% on any isoform</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -1388,7 +1390,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Most flagged isoform</t>
+          <t>Project benchmark: most flagged isoform</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1400,7 +1402,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Compounds &gt;50% on that isoform</t>
+          <t>Project benchmark: &gt;50% on that isoform</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -1428,172 +1430,185 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Repeat of the poorly recovered sample; signed report after the repeat and biology memo review.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+          <t>Poorly recovered sample repeat; reconcile outstanding compound rows and benchmark counts before signed report release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark counts describe the project screening set and cannot be reconstructed from this partial interim compound table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>BW26_0401</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Elvarmere Biosciences AB</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Compounds tested</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>40</v>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>BW26_0401</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Series / chemotype</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Elvarmere pyrrolopyridine series 05 (Pyrrolopyridine)</t>
+          <t>Elvarmere Biosciences AB</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Assays</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>CYP inhibition panel (1A2/2C9/2C19/2D6/3A4) at 10 µM</t>
-        </is>
+          <t>Compounds tested</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Turnaround (calendar days)</t>
+          <t>Series / chemotype</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Elvarmere pyrrolopyridine series 05 (Pyrrolopyridine)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Assays</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>GBP 14,300</t>
+          <t>CYP inhibition panel (1A2/2C9/2C19/2D6/3A4) at 10 µM</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CYP1A2 &gt;50% inhibition @10 µM</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>8</v>
+          <t>Turnaround (calendar days)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CYP2C9 &gt;50% inhibition @10 µM</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>9</v>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>GBP 14,300</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CYP2C19 &gt;50% inhibition @10 µM</t>
+          <t>CYP1A2 &gt;50% inhibition @10 µM</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CYP2D6 &gt;50% inhibition @10 µM</t>
+          <t>CYP2C9 &gt;50% inhibition @10 µM</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CYP3A4 &gt;50% inhibition @10 µM</t>
+          <t>CYP2C19 &gt;50% inhibition @10 µM</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Compounds with any CYP &gt;50%</t>
+          <t>CYP2D6 &gt;50% inhibition @10 µM</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>CYP3A4 &gt;50% inhibition @10 µM</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Compounds with any CYP &gt;50%</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Ketoconazole (3A4) IC50 (µM)</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B27" s="2" t="n">
         <v>0.035</v>
       </c>
     </row>

</xml_diff>